<commit_message>
fix: seed available resource links in modules
</commit_message>
<xml_diff>
--- a/BE/app/scripts/BCG_Onboarding_Quick_Reference_Developer_Handoff.xlsx
+++ b/BE/app/scripts/BCG_Onboarding_Quick_Reference_Developer_Handoff.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nagarro.sharepoint.com/teams/bcg/Shared Documents/GSD-2026/Initiatives/Onboarding Portal/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu\home\harshit\projects\internal\onboarding-module-repo\BE-AILearningApp\BE\app\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F25A8A6-9AAC-43CD-A37C-C135CEDF5F80}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7373EAE0-5678-44E9-AF9E-DED9E4217F90}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="115">
   <si>
     <t>Quick Reference Content by Module</t>
   </si>
@@ -287,9 +287,6 @@
     <t>Access SAP Concur to create, submit and track your reimbursement claims.</t>
   </si>
   <si>
-    <t>Direct clickable link | URL TO BE ADDED</t>
-  </si>
-  <si>
     <t>Open SAP Concur directly using the URL entered in this cell.</t>
   </si>
   <si>
@@ -360,13 +357,37 @@
   </si>
   <si>
     <t>Explain the flow without adding a separate linked guide.</t>
+  </si>
+  <si>
+    <t>https://nagarro.sharepoint.com/:x:/r/sites/BCGIndiaGSD/Shared%20Documents/General/Resource%20Master%20Sheet_GSD.xlsx?d=wc41d688d708244cb98792f260ec08760&amp;csf=1&amp;web=1&amp;e=vnsM7j</t>
+  </si>
+  <si>
+    <t>https://teams.microsoft.com/l/team/19%3Adce3bde1d57243f4b1e7cad89e6beae7%40thread.tacv2/conversations?groupId=a70f178a-b822-46d5-838b-e075ee71f781&amp;tenantId=a45fe71a-f480-4e42-ad5e-aff33165aa35</t>
+  </si>
+  <si>
+    <t>windowsvirtualdesktop@bcg.com ; Gali.venkata@bcg.com</t>
+  </si>
+  <si>
+    <t>https://nagarro.sharepoint.com/teams/bcg/Shared Documents/GSD-2026/Initiatives/Onboarding Portal/../../../../../../sites/Ginger/OperatingManual/Operating%20manual%20for%20Ginger/Timesheet.aspx?xsdata=MDV8MDJ8fDVhZGFmMWE5ZDkxNjRiZDE0ZGIzMDhkZWU5NDE3ZjBjfGE0NWZlNzFhZjQ4MDRlNDJhZDVlYWZmMzMxNjVhYTM1fDB8MHw2MzkyMDQ2NjQ2NDY4NDc5MjN8VW5rbm93bnxWR1ZoYlhOVFpXTjFjbWwwZVZObGNuWnBZMlY4ZXlKRFFTSTZJbFJsWVcxelgwRlVVRk5sY25acFkyVmZVMUJQVEU5R0lpd2lWaUk2SWpBdU1DNHdNREF3SWl3aVVDSTZJbGRwYmpNeUlpd2lRVTRpT2lKUGRHaGxjaUlzSWxkVUlqb3hNWDA9fDF8TDJOb1lYUnpMekU1T2pZME1XWTROMlV3TFRFMFlXWXRORGcwTmkwNVpqVXlMV1U0T1RFeU56WTFZVFUxTTE4M1pETm1NVGszT1Mxak1UZzRMVFExTWpndE9USTRNaTA0WWpjNFkyUXdZMkpoWkRCQWRXNXhMbWRpYkM1emNHRmpaWE12YldWemMyRm5aWE12TVRjNE5EZzJPVFkyTXpRMU5BPT18MmFjZmNiZWFlNTc2NGNiM2FmODEwOGRlZTk0MTdmMGJ8Yjg5YmFmNWMzZDg3NGUzOWJhYWM1MDZlY2IyZDM2Yzg%3D&amp;sdata=QlhYSTRJSHhyeU5nWjg2ZktvSURsWHNRdkpadWpBd2dVcTZsV2FJOEdqYz0%3D&amp;ovuser=a45fe71a-f480-4e42-ad5e-aff33165aa35%2Cmonika.singh01%40nagarro.com&amp;TeamsCID=e3681ad9-cc24-41b7-a99e-ade0f895ce46&amp;OR=Teams-HL&amp;CT=1784869701297&amp;clickparams=eyJBcHBOYW1lIjoiVGVhbXMtRGVza3RvcCIsIkFwcFZlcnNpb24iOiI0OS8yNjA2MTExODIxNiIsIkhhc0ZlZGVyYXRlZFVzZXIiOmZhbHNlfQ%3D%3D</t>
+  </si>
+  <si>
+    <t>https://nagarro.sharepoint.com/teams/bcg/Shared Documents/GSD-2026/Initiatives/Onboarding Portal/../../../../../../sites/BCGIndiaGSD/Lists/BCG%20GSD%20Leave%20Calendar/LeaveSubmission.aspx?viewid=69d58e5e%2D0783%2D40c4%2Db57f%2Df84d077ad8e3&amp;env=WebViewList&amp;OR=Teams%2DHL&amp;CT=1774244885641&amp;clickparams=eyJBcHBOYW1lIjoiVGVhbXMtRGVza3RvcCIsIkFwcFZlcnNpb24iOiI0OS8yNjAyMTIxNTEyMyJ9&amp;xsdata=MDV8MDJ8fGQxN2RiNjcxYjM3NDQxNzU1MDZiMDhkZWQxY2ExMzg4fGE0NWZlNzFhZjQ4MDRlNDJhZDVlYWZmMzMxNjVhYTM1fDB8MHw2MzkxNzg4NjI5NzQ0ODg2ODN8VW5rbm93bnxWR1ZoYlhOVFpXTjFjbWwwZVZObGNuWnBZMlY4ZXlKRFFTSTZJbFJsWVcxelgwRlVVRk5sY25acFkyVmZVMUJQVEU5R0lpd2lWaUk2SWpBdU1DNHdNREF3SWl3aVVDSTZJbGRwYmpNeUlpd2lRVTRpT2lKUGRHaGxjaUlzSWxkVUlqb3hNWDA9fDF8TDNSbFlXMXpMekU1T21SalpUTmlaR1V4WkRVM01qUXpaalJpTVdVM1kyRmtPRGxsTm1KbFlXVTNRSFJvY21WaFpDNTBZV04yTWk5amFHRnVibVZzY3k4eE9UcGtZMlV6WW1SbE1XUTFOekkwTTJZMFlqRmxOMk5oWkRnNVpUWmlaV0ZsTjBCMGFISmxZV1F1ZEdGamRqSXZiV1Z6YzJGblpYTXZNVGM0TWpJNE9UUTVOVFV6TVE9PXw2MzAwMWQ5OTkzZTM0ZDY1ZjUyZDA4ZGVkMWNhMTM4N3xmM2E5YjA4MWU4NGI0N2U2YWI4MjQ1MGMxOTQ0MDUxYQ%3D%3D&amp;sdata=cTMvNzhkWFBEZXFiQ3BwdjBiWjNvNFhDamlaeE43aGRDWHpyTnZsQ0tOdz0%3D&amp;ovuser=a45fe71a-f480-4e42-ad5e-aff33165aa35%2Cmonika.singh01%40nagarro.com</t>
+  </si>
+  <si>
+    <t>https://nagarro.sharepoint.com/teams/bcg/Shared Documents/GSD-2026/Initiatives/Onboarding Portal/../../../../../../:f:/r/sites/BCGIndiaGSD/Shared%20Documents/General/Holiday%20Calendar%202026?csf=1&amp;web=1&amp;e=e9bySe</t>
+  </si>
+  <si>
+    <t>https://eu2.concursolutions.com/home</t>
+  </si>
+  <si>
+    <t>https://nagarro.sharepoint.com/:v:/r/sites/BCGIndiaGSD/Shared%20Documents/General/SAP%20Concur%20reimbursements%20process/SAP%20Concur%20reimbursements-process%20Recording.mp4?csf=1&amp;web=1&amp;e=n5KAge</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <name val="Carlito"/>
@@ -393,6 +414,12 @@
       <b/>
       <sz val="11"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Carlito"/>
     </font>
   </fonts>
@@ -458,10 +485,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -496,8 +524,13 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
@@ -700,7 +733,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:G37"/>
-  <sheetFormatPr defaultRowHeight="14.1"/>
+  <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
@@ -711,7 +744,7 @@
     <col min="7" max="7" width="48" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="20.100000000000001" customHeight="1">
+    <row r="1" spans="1:7" ht="20.149999999999999" customHeight="1">
       <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
@@ -722,7 +755,7 @@
       <c r="F1" s="10"/>
       <c r="G1" s="10"/>
     </row>
-    <row r="2" spans="1:7" ht="14.45">
+    <row r="2" spans="1:7" ht="14.5">
       <c r="A2" s="11" t="s">
         <v>1</v>
       </c>
@@ -756,7 +789,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="30.6" customHeight="1">
+    <row r="5" spans="1:7" ht="30.65" customHeight="1">
       <c r="A5" s="4">
         <v>1</v>
       </c>
@@ -779,7 +812,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="30.6" customHeight="1">
+    <row r="6" spans="1:7" ht="30.65" customHeight="1">
       <c r="A6" s="4">
         <v>1</v>
       </c>
@@ -802,7 +835,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="30.6" customHeight="1">
+    <row r="7" spans="1:7" ht="30.65" customHeight="1">
       <c r="A7" s="4">
         <v>1</v>
       </c>
@@ -818,14 +851,14 @@
       <c r="E7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>19</v>
+      <c r="F7" s="12" t="s">
+        <v>107</v>
       </c>
       <c r="G7" s="2" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="30.6" customHeight="1">
+    <row r="8" spans="1:7" ht="30.65" customHeight="1">
       <c r="A8" s="4">
         <v>1</v>
       </c>
@@ -841,14 +874,14 @@
       <c r="E8" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>19</v>
+      <c r="F8" s="12" t="s">
+        <v>108</v>
       </c>
       <c r="G8" s="2" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="30.6" customHeight="1">
+    <row r="9" spans="1:7" ht="30.65" customHeight="1">
       <c r="A9" s="4">
         <v>1</v>
       </c>
@@ -871,7 +904,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="30.6" customHeight="1">
+    <row r="10" spans="1:7" ht="30.65" customHeight="1">
       <c r="A10" s="5">
         <v>2</v>
       </c>
@@ -894,7 +927,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="30.6" customHeight="1">
+    <row r="11" spans="1:7" ht="30.65" customHeight="1">
       <c r="A11" s="5">
         <v>2</v>
       </c>
@@ -917,7 +950,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="30.6" customHeight="1">
+    <row r="12" spans="1:7" ht="30.65" customHeight="1">
       <c r="A12" s="5">
         <v>2</v>
       </c>
@@ -940,7 +973,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="30.6" customHeight="1">
+    <row r="13" spans="1:7" ht="30.65" customHeight="1">
       <c r="A13" s="5">
         <v>2</v>
       </c>
@@ -957,13 +990,13 @@
         <v>37</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>19</v>
+        <v>109</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="30.6" customHeight="1">
+    <row r="14" spans="1:7" ht="30.65" customHeight="1">
       <c r="A14" s="5">
         <v>2</v>
       </c>
@@ -986,7 +1019,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="30.6" customHeight="1">
+    <row r="15" spans="1:7" ht="30.65" customHeight="1">
       <c r="A15" s="5">
         <v>2</v>
       </c>
@@ -1009,7 +1042,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="30.6" customHeight="1">
+    <row r="16" spans="1:7" ht="30.65" customHeight="1">
       <c r="A16" s="6">
         <v>3</v>
       </c>
@@ -1032,7 +1065,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="30.6" customHeight="1">
+    <row r="17" spans="1:7" ht="30.65" customHeight="1">
       <c r="A17" s="6">
         <v>3</v>
       </c>
@@ -1048,14 +1081,14 @@
       <c r="E17" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>19</v>
+      <c r="F17" s="13" t="s">
+        <v>110</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="30.6" customHeight="1">
+    <row r="18" spans="1:7" ht="30.65" customHeight="1">
       <c r="A18" s="6">
         <v>3</v>
       </c>
@@ -1071,14 +1104,14 @@
       <c r="E18" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>19</v>
+      <c r="F18" s="12" t="s">
+        <v>111</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="30.6" customHeight="1">
+    <row r="19" spans="1:7" ht="30.65" customHeight="1">
       <c r="A19" s="6">
         <v>3</v>
       </c>
@@ -1094,14 +1127,14 @@
       <c r="E19" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>19</v>
+      <c r="F19" s="12" t="s">
+        <v>112</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="30.6" customHeight="1">
+    <row r="20" spans="1:7" ht="30.65" customHeight="1">
       <c r="A20" s="6">
         <v>3</v>
       </c>
@@ -1124,7 +1157,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="30.6" customHeight="1">
+    <row r="21" spans="1:7" ht="30.65" customHeight="1">
       <c r="A21" s="6">
         <v>3</v>
       </c>
@@ -1147,7 +1180,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="30.6" customHeight="1">
+    <row r="22" spans="1:7" ht="30.65" customHeight="1">
       <c r="A22" s="7">
         <v>4</v>
       </c>
@@ -1170,7 +1203,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="30.6" customHeight="1">
+    <row r="23" spans="1:7" ht="30.65" customHeight="1">
       <c r="A23" s="7">
         <v>4</v>
       </c>
@@ -1193,7 +1226,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="30.6" customHeight="1">
+    <row r="24" spans="1:7" ht="30.65" customHeight="1">
       <c r="A24" s="7">
         <v>4</v>
       </c>
@@ -1216,7 +1249,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="30.6" customHeight="1">
+    <row r="25" spans="1:7" ht="30.65" customHeight="1">
       <c r="A25" s="7">
         <v>4</v>
       </c>
@@ -1239,7 +1272,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="30.6" customHeight="1">
+    <row r="26" spans="1:7" ht="30.65" customHeight="1">
       <c r="A26" s="7">
         <v>4</v>
       </c>
@@ -1262,7 +1295,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="30.6" customHeight="1">
+    <row r="27" spans="1:7" ht="30.65" customHeight="1">
       <c r="A27" s="7">
         <v>4</v>
       </c>
@@ -1285,7 +1318,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="30.6" customHeight="1">
+    <row r="28" spans="1:7" ht="30.65" customHeight="1">
       <c r="A28" s="8">
         <v>5</v>
       </c>
@@ -1308,7 +1341,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="30.6" customHeight="1">
+    <row r="29" spans="1:7" ht="30.65" customHeight="1">
       <c r="A29" s="8">
         <v>5</v>
       </c>
@@ -1324,14 +1357,14 @@
       <c r="E29" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="F29" s="2" t="s">
+      <c r="F29" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="G29" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="G29" s="2" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="30" spans="1:7" ht="30.6" customHeight="1">
+    </row>
+    <row r="30" spans="1:7" ht="30.65" customHeight="1">
       <c r="A30" s="8">
         <v>5</v>
       </c>
@@ -1342,19 +1375,19 @@
         <v>3</v>
       </c>
       <c r="D30" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="E30" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E30" s="2" t="s">
+      <c r="F30" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="G30" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="F30" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="31" spans="1:7" ht="30.6" customHeight="1">
+    </row>
+    <row r="31" spans="1:7" ht="30.65" customHeight="1">
       <c r="A31" s="8">
         <v>5</v>
       </c>
@@ -1365,19 +1398,19 @@
         <v>4</v>
       </c>
       <c r="D31" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="E31" s="2" t="s">
         <v>88</v>
-      </c>
-      <c r="E31" s="2" t="s">
-        <v>89</v>
       </c>
       <c r="F31" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G31" s="2" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="32" spans="1:7" ht="30.6" customHeight="1">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" ht="30.65" customHeight="1">
       <c r="A32" s="8">
         <v>5</v>
       </c>
@@ -1388,10 +1421,10 @@
         <v>5</v>
       </c>
       <c r="D32" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="E32" s="2" t="s">
         <v>91</v>
-      </c>
-      <c r="E32" s="2" t="s">
-        <v>92</v>
       </c>
       <c r="F32" s="2" t="s">
         <v>12</v>
@@ -1400,90 +1433,90 @@
         <v>13</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="30.6" customHeight="1">
+    <row r="33" spans="1:7" ht="30.65" customHeight="1">
       <c r="A33" s="9">
         <v>6</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C33" s="3">
         <v>1</v>
       </c>
       <c r="D33" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="E33" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E33" s="2" t="s">
+      <c r="F33" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G33" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F33" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G33" s="2" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="34" spans="1:7" ht="30.6" customHeight="1">
+    </row>
+    <row r="34" spans="1:7" ht="30.65" customHeight="1">
       <c r="A34" s="9">
         <v>6</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C34" s="3">
         <v>2</v>
       </c>
       <c r="D34" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="E34" s="2" t="s">
+      <c r="F34" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="F34" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="2" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="35" spans="1:7" ht="30.6" customHeight="1">
+    </row>
+    <row r="35" spans="1:7" ht="30.65" customHeight="1">
       <c r="A35" s="9">
         <v>6</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C35" s="3">
         <v>3</v>
       </c>
       <c r="D35" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="E35" s="2" t="s">
         <v>100</v>
-      </c>
-      <c r="E35" s="2" t="s">
-        <v>101</v>
       </c>
       <c r="F35" s="2" t="s">
         <v>19</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="36" spans="1:7" ht="30.6" customHeight="1">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" ht="30.65" customHeight="1">
       <c r="A36" s="9">
         <v>6</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C36" s="3">
         <v>4</v>
       </c>
       <c r="D36" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="E36" s="2" t="s">
         <v>103</v>
-      </c>
-      <c r="E36" s="2" t="s">
-        <v>104</v>
       </c>
       <c r="F36" s="2" t="s">
         <v>12</v>
@@ -1492,27 +1525,27 @@
         <v>13</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="30.6" customHeight="1">
+    <row r="37" spans="1:7" ht="30.65" customHeight="1">
       <c r="A37" s="9">
         <v>6</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C37" s="3">
         <v>5</v>
       </c>
       <c r="D37" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="E37" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="E37" s="2" t="s">
+      <c r="F37" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G37" s="2" t="s">
         <v>106</v>
-      </c>
-      <c r="F37" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="G37" s="2" t="s">
-        <v>107</v>
       </c>
     </row>
   </sheetData>
@@ -1520,7 +1553,7 @@
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
   </mergeCells>
-  <conditionalFormatting sqref="F5:F37">
+  <conditionalFormatting sqref="F5:F16 F18:F37">
     <cfRule type="expression" dxfId="1" priority="1">
       <formula>ISNUMBER(SEARCH("URL TO BE ADDED",F5))</formula>
     </cfRule>
@@ -1528,25 +1561,23 @@
       <formula>ISNUMBER(SEARCH("Display directly",F5))</formula>
     </cfRule>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="F7" r:id="rId1" xr:uid="{E298EA24-BE18-4CFA-B78D-56DDC94EAF57}"/>
+    <hyperlink ref="F8" r:id="rId2" xr:uid="{007530AE-E7CD-4D15-AB00-98B130FD3D4B}"/>
+    <hyperlink ref="F17" r:id="rId3" display="https://nagarro.sharepoint.com/sites/Ginger/OperatingManual/Operating%20manual%20for%20Ginger/Timesheet.aspx?xsdata=MDV8MDJ8fDVhZGFmMWE5ZDkxNjRiZDE0ZGIzMDhkZWU5NDE3ZjBjfGE0NWZlNzFhZjQ4MDRlNDJhZDVlYWZmMzMxNjVhYTM1fDB8MHw2MzkyMDQ2NjQ2NDY4NDc5MjN8VW5rbm93bnxWR1ZoYlhOVFpXTjFjbWwwZVZObGNuWnBZMlY4ZXlKRFFTSTZJbFJsWVcxelgwRlVVRk5sY25acFkyVmZVMUJQVEU5R0lpd2lWaUk2SWpBdU1DNHdNREF3SWl3aVVDSTZJbGRwYmpNeUlpd2lRVTRpT2lKUGRHaGxjaUlzSWxkVUlqb3hNWDA9fDF8TDJOb1lYUnpMekU1T2pZME1XWTROMlV3TFRFMFlXWXRORGcwTmkwNVpqVXlMV1U0T1RFeU56WTFZVFUxTTE4M1pETm1NVGszT1Mxak1UZzRMVFExTWpndE9USTRNaTA0WWpjNFkyUXdZMkpoWkRCQWRXNXhMbWRpYkM1emNHRmpaWE12YldWemMyRm5aWE12TVRjNE5EZzJPVFkyTXpRMU5BPT18MmFjZmNiZWFlNTc2NGNiM2FmODEwOGRlZTk0MTdmMGJ8Yjg5YmFmNWMzZDg3NGUzOWJhYWM1MDZlY2IyZDM2Yzg%3D&amp;sdata=QlhYSTRJSHhyeU5nWjg2ZktvSURsWHNRdkpadWpBd2dVcTZsV2FJOEdqYz0%3D&amp;ovuser=a45fe71a-f480-4e42-ad5e-aff33165aa35%2Cmonika.singh01%40nagarro.com&amp;TeamsCID=e3681ad9-cc24-41b7-a99e-ade0f895ce46&amp;OR=Teams-HL&amp;CT=1784869701297&amp;clickparams=eyJBcHBOYW1lIjoiVGVhbXMtRGVza3RvcCIsIkFwcFZlcnNpb24iOiI0OS8yNjA2MTExODIxNiIsIkhhc0ZlZGVyYXRlZFVzZXIiOmZhbHNlfQ%3D%3D" xr:uid="{D1A73D23-A764-4CD1-9979-4BC86B090CFB}"/>
+    <hyperlink ref="F18" r:id="rId4" display="https://nagarro.sharepoint.com/teams/bcg/Shared Documents/GSD-2026/Initiatives/Onboarding Portal/../../../../../../sites/BCGIndiaGSD/Lists/BCG%20GSD%20Leave%20Calendar/LeaveSubmission.aspx?viewid=69d58e5e%2D0783%2D40c4%2Db57f%2Df84d077ad8e3&amp;env=WebViewList&amp;OR=Teams%2DHL&amp;CT=1774244885641&amp;clickparams=eyJBcHBOYW1lIjoiVGVhbXMtRGVza3RvcCIsIkFwcFZlcnNpb24iOiI0OS8yNjAyMTIxNTEyMyJ9&amp;xsdata=MDV8MDJ8fGQxN2RiNjcxYjM3NDQxNzU1MDZiMDhkZWQxY2ExMzg4fGE0NWZlNzFhZjQ4MDRlNDJhZDVlYWZmMzMxNjVhYTM1fDB8MHw2MzkxNzg4NjI5NzQ0ODg2ODN8VW5rbm93bnxWR1ZoYlhOVFpXTjFjbWwwZVZObGNuWnBZMlY4ZXlKRFFTSTZJbFJsWVcxelgwRlVVRk5sY25acFkyVmZVMUJQVEU5R0lpd2lWaUk2SWpBdU1DNHdNREF3SWl3aVVDSTZJbGRwYmpNeUlpd2lRVTRpT2lKUGRHaGxjaUlzSWxkVUlqb3hNWDA9fDF8TDNSbFlXMXpMekU1T21SalpUTmlaR1V4WkRVM01qUXpaalJpTVdVM1kyRmtPRGxsTm1KbFlXVTNRSFJvY21WaFpDNTBZV04yTWk5amFHRnVibVZzY3k4eE9UcGtZMlV6WW1SbE1XUTFOekkwTTJZMFlqRmxOMk5oWkRnNVpUWmlaV0ZsTjBCMGFISmxZV1F1ZEdGamRqSXZiV1Z6YzJGblpYTXZNVGM0TWpJNE9UUTVOVFV6TVE9PXw2MzAwMWQ5OTkzZTM0ZDY1ZjUyZDA4ZGVkMWNhMTM4N3xmM2E5YjA4MWU4NGI0N2U2YWI4MjQ1MGMxOTQ0MDUxYQ%3D%3D&amp;sdata=cTMvNzhkWFBEZXFiQ3BwdjBiWjNvNFhDamlaeE43aGRDWHpyTnZsQ0tOdz0%3D&amp;ovuser=a45fe71a-f480-4e42-ad5e-aff33165aa35%2Cmonika.singh01%40nagarro.com" xr:uid="{4D52B546-9F92-40ED-B3C1-310F3848EACE}"/>
+    <hyperlink ref="F19" r:id="rId5" xr:uid="{12AF9FCC-92E0-4EFC-B04E-1BA1E695B10F}"/>
+    <hyperlink ref="F29" r:id="rId6" xr:uid="{5F5B1632-87EB-41DE-9F64-E312A3801378}"/>
+    <hyperlink ref="F30" r:id="rId7" xr:uid="{B7AB1F5A-100F-4B1C-AEED-615CD98ECDCD}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId8"/>
   </tableParts>
 </worksheet>
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="11f7c52c-c25f-4875-906f-6d84de8f56d5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4aef3c27-fe4d-4946-b9c8-b2b267a34f77">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F78ACF99C79F2B49AC9F2C200D2B2466" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="0d9878a2c3a28fa6d6619464a0a4cdaa">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4aef3c27-fe4d-4946-b9c8-b2b267a34f77" xmlns:ns3="11f7c52c-c25f-4875-906f-6d84de8f56d5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f4945d78a66e60d2963e961e4725d98d" ns2:_="" ns3:_="">
     <xsd:import namespace="4aef3c27-fe4d-4946-b9c8-b2b267a34f77"/>
@@ -1807,6 +1838,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="11f7c52c-c25f-4875-906f-6d84de8f56d5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="4aef3c27-fe4d-4946-b9c8-b2b267a34f77">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -1817,13 +1859,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35A8BA5A-81D0-46F8-BF19-2FA56F22DDEB}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A18C3BA-775B-499D-AC88-4A888328CE5C}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="4aef3c27-fe4d-4946-b9c8-b2b267a34f77"/>
+    <ds:schemaRef ds:uri="11f7c52c-c25f-4875-906f-6d84de8f56d5"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2A18C3BA-775B-499D-AC88-4A888328CE5C}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{35A8BA5A-81D0-46F8-BF19-2FA56F22DDEB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="11f7c52c-c25f-4875-906f-6d84de8f56d5"/>
+    <ds:schemaRef ds:uri="4aef3c27-fe4d-4946-b9c8-b2b267a34f77"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEECC09-8456-42AF-AFB6-D25367CCC9EE}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{4FEECC09-8456-42AF-AFB6-D25367CCC9EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>